<commit_message>
job-tracker: remove ASIO on Eileen's confirmation
PR #24 kept this row against the letter of the request, because it was a real
application rather than an unactioned lead -- applied 2026-09-09, status
Withdrawn -- and deleting application history to fix a missing favicon was
the wrong trade to make unilaterally. Raised, confirmed, removed.

Out of job-applications.xlsx, the source of truth, so regenerating cannot
bring it back. 84 entries -> 83; Withdrawn falls from 8 to 7.

Every remaining company now has a cached logo: 75 referenced domains, 75
files, nothing missing and nothing orphaned. The initials fallback in
renderLogo() stays -- it is what covers a company added to the sheet before
its logo is fetched -- but nothing on the page currently needs it.

Verified at 1280px with lazy loading forced off so the audit was real: 83
rows, zero initials tiles, no ASIO, no horizontal overflow.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -1088,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC89"/>
+  <dimension ref="A1:AC88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="31" min="1" max="1"/>
@@ -6591,12 +6591,12 @@
     <row r="83" ht="15.75" customHeight="1" s="31">
       <c r="A83" s="32" t="inlineStr">
         <is>
-          <t>australian secruity intelligence organisation asio</t>
+          <t>accenture</t>
         </is>
       </c>
       <c r="B83" s="32" t="inlineStr">
         <is>
-          <t>intelligence development program itelligence analyst</t>
+          <t>graduate analyst technology</t>
         </is>
       </c>
       <c r="C83" s="32" t="inlineStr">
@@ -6606,16 +6606,13 @@
       </c>
       <c r="D83" s="32" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="F83" s="6" t="n">
-        <v>46258</v>
-      </c>
-      <c r="G83" s="6" t="n">
-        <v>46274</v>
-      </c>
-      <c r="H83" s="13" t="inlineStr">
+        <v>46264</v>
+      </c>
+      <c r="H83" s="32" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
@@ -6627,79 +6624,72 @@
       </c>
       <c r="P83" s="6" t="inlineStr">
         <is>
-          <t>ongoing</t>
-        </is>
-      </c>
-      <c r="T83" s="32" t="inlineStr">
-        <is>
-          <t>100425 - 125060</t>
+          <t>1/19/2027 - 7/13/2027</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>70000-80000</t>
         </is>
       </c>
       <c r="U83" s="7" t="inlineStr">
         <is>
-          <t>5-50</t>
+          <t>1-45</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="31">
       <c r="A84" s="32" t="inlineStr">
         <is>
-          <t>accenture</t>
-        </is>
-      </c>
-      <c r="B84" s="32" t="inlineStr">
-        <is>
-          <t>graduate analyst technology</t>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>business data analyst project intern (GBS)</t>
         </is>
       </c>
       <c r="C84" s="32" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D84" s="32" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="F84" s="6" t="n">
-        <v>46264</v>
-      </c>
-      <c r="H84" s="32" t="inlineStr">
+        <v>46387</v>
+      </c>
+      <c r="G84" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H84" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="M84" s="32" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="P84" s="6" t="inlineStr">
-        <is>
-          <t>1/19/2027 - 7/13/2027</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="T84" t="inlineStr">
         <is>
-          <t>70000-80000</t>
-        </is>
-      </c>
-      <c r="U84" s="7" t="inlineStr">
-        <is>
-          <t>1-45</t>
+          <t>2000-5000 per month</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1" s="31">
       <c r="A85" s="32" t="inlineStr">
         <is>
-          <t>tiktok</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>business data analyst project intern (GBS)</t>
+          <t>Didi</t>
+        </is>
+      </c>
+      <c r="B85" s="32" t="inlineStr">
+        <is>
+          <t>operations intern</t>
         </is>
       </c>
       <c r="C85" s="32" t="inlineStr">
@@ -6711,38 +6701,25 @@
         <is>
           <t>NSW</t>
         </is>
-      </c>
-      <c r="F85" s="6" t="n">
-        <v>46387</v>
       </c>
       <c r="G85" s="34" t="n">
         <v>46277</v>
       </c>
-      <c r="H85" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
       <c r="M85" s="32" t="inlineStr">
         <is>
           <t>Applied</t>
-        </is>
-      </c>
-      <c r="T85" t="inlineStr">
-        <is>
-          <t>2000-5000 per month</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="32" t="inlineStr">
         <is>
-          <t>Didi</t>
-        </is>
-      </c>
-      <c r="B86" s="32" t="inlineStr">
-        <is>
-          <t>operations intern</t>
+          <t>tencent</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Game Reaserch Development intern, engine reasearch</t>
         </is>
       </c>
       <c r="C86" s="32" t="inlineStr">
@@ -6767,12 +6744,12 @@
     <row r="87">
       <c r="A87" s="32" t="inlineStr">
         <is>
-          <t>tencent</t>
+          <t>apple</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Game Reaserch Development intern, engine reasearch</t>
+          <t>information systems and technology</t>
         </is>
       </c>
       <c r="C87" s="32" t="inlineStr">
@@ -6797,12 +6774,12 @@
     <row r="88">
       <c r="A88" s="32" t="inlineStr">
         <is>
-          <t>apple</t>
+          <t>SAP</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>information systems and technology</t>
+          <t>student training and totation program intern</t>
         </is>
       </c>
       <c r="C88" s="32" t="inlineStr">
@@ -6812,7 +6789,7 @@
       </c>
       <c r="D88" s="32" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="G88" s="34" t="n">
@@ -6823,37 +6800,7 @@
           <t>Applied</t>
         </is>
       </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="32" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>student training and totation program intern</t>
-        </is>
-      </c>
-      <c r="C89" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D89" s="32" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="G89" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="M89" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="R89" t="inlineStr">
+      <c r="R88" t="inlineStr">
         <is>
           <t>2 years</t>
         </is>

</xml_diff>

<commit_message>
jobs: mark confirmed rejections, add AusDN and FDM, remove never-applied rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6LghyMTCB4an1gFe21ULf
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Answers" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$AC$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$AC$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Answers'!$A$1:$E$40</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1088,7 +1088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC88"/>
+  <dimension ref="A1:AC56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="20" customWidth="1" style="31" min="1" max="1"/>
@@ -1516,7 +1516,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="13" t="inlineStr">
         <is>
-          <t>Applied</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="N5" s="13" t="n"/>
@@ -3662,12 +3662,12 @@
     <row r="35" ht="18" customHeight="1" s="31">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>amazon</t>
+          <t>city of gold coast</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Graduate Brand Analyst,</t>
+          <t>digital and data</t>
         </is>
       </c>
       <c r="C35" s="13" t="inlineStr">
@@ -3677,13 +3677,11 @@
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E35" s="13" t="n"/>
-      <c r="F35" s="14" t="n">
-        <v>46147</v>
-      </c>
+      <c r="F35" s="13" t="n"/>
       <c r="G35" s="13" t="n"/>
       <c r="H35" s="13" t="inlineStr">
         <is>
@@ -3694,15 +3692,17 @@
       <c r="J35" s="13" t="n"/>
       <c r="K35" s="13" t="n"/>
       <c r="L35" s="13" t="n"/>
-      <c r="M35" s="13" t="n"/>
+      <c r="M35" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
       <c r="N35" s="13" t="n"/>
       <c r="O35" s="13" t="n"/>
-      <c r="P35" s="14" t="n">
-        <v>46204</v>
-      </c>
+      <c r="P35" s="13" t="n"/>
       <c r="Q35" s="17" t="n"/>
       <c r="R35" s="18">
-        <f>IF(AND(P38&lt;&gt;"",Q38&lt;&gt;""),Q38-P38,"")</f>
+        <f>IF(AND(P44&lt;&gt;"",Q44&lt;&gt;""),Q44-P44,"")</f>
         <v/>
       </c>
       <c r="S35" s="13" t="n"/>
@@ -3720,18 +3720,22 @@
     <row r="36" ht="18" customHeight="1" s="31">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>anz</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="n"/>
+          <t>commbank</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>tech ai engineering data science &amp; ai</t>
+        </is>
+      </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E36" s="13" t="n"/>
@@ -3746,17 +3750,27 @@
       <c r="J36" s="13" t="n"/>
       <c r="K36" s="13" t="n"/>
       <c r="L36" s="13" t="n"/>
-      <c r="M36" s="13" t="n"/>
+      <c r="M36" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
       <c r="N36" s="13" t="n"/>
       <c r="O36" s="13" t="n"/>
-      <c r="P36" s="13" t="n"/>
+      <c r="P36" s="14" t="n">
+        <v>46349</v>
+      </c>
       <c r="Q36" s="17" t="n"/>
       <c r="R36" s="18">
-        <f>IF(AND(P39&lt;&gt;"",Q39&lt;&gt;""),Q39-P39,"")</f>
+        <f>IF(AND(P45&lt;&gt;"",Q45&lt;&gt;""),Q45-P45,"")</f>
         <v/>
       </c>
       <c r="S36" s="13" t="n"/>
-      <c r="T36" s="13" t="n"/>
+      <c r="T36" s="13" t="inlineStr">
+        <is>
+          <t>65k</t>
+        </is>
+      </c>
       <c r="U36" s="20" t="n"/>
       <c r="V36" s="13" t="n"/>
       <c r="W36" s="13" t="n"/>
@@ -3770,12 +3784,12 @@
     <row r="37" ht="18" customHeight="1" s="31">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>bcg</t>
+          <t>eightcap</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>consulting</t>
+          <t>operations analyst</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
@@ -3789,9 +3803,7 @@
         </is>
       </c>
       <c r="E37" s="13" t="n"/>
-      <c r="F37" s="14" t="n">
-        <v>46085</v>
-      </c>
+      <c r="F37" s="13" t="n"/>
       <c r="G37" s="13" t="n"/>
       <c r="H37" s="13" t="inlineStr">
         <is>
@@ -3802,13 +3814,17 @@
       <c r="J37" s="13" t="n"/>
       <c r="K37" s="13" t="n"/>
       <c r="L37" s="13" t="n"/>
-      <c r="M37" s="13" t="n"/>
+      <c r="M37" s="13" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
       <c r="N37" s="13" t="n"/>
       <c r="O37" s="13" t="n"/>
       <c r="P37" s="13" t="n"/>
       <c r="Q37" s="17" t="n"/>
       <c r="R37" s="18">
-        <f>IF(AND(P40&lt;&gt;"",Q40&lt;&gt;""),Q40-P40,"")</f>
+        <f>IF(AND(P48&lt;&gt;"",Q48&lt;&gt;""),Q48-P48,"")</f>
         <v/>
       </c>
       <c r="S37" s="13" t="n"/>
@@ -3826,12 +3842,12 @@
     <row r="38" ht="18" customHeight="1" s="31">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>bloomberg</t>
+          <t>loreal</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>analytics &amp; sales</t>
+          <t>Management Trainee Program – Data &amp; Analytics Stream</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -3841,14 +3857,16 @@
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E38" s="13" t="n"/>
       <c r="F38" s="14" t="n">
-        <v>46266</v>
-      </c>
-      <c r="G38" s="13" t="n"/>
+        <v>46093</v>
+      </c>
+      <c r="G38" s="33" t="n">
+        <v>46277</v>
+      </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3858,28 +3876,30 @@
       <c r="J38" s="13" t="n"/>
       <c r="K38" s="13" t="n"/>
       <c r="L38" s="13" t="n"/>
-      <c r="M38" s="13" t="n"/>
+      <c r="M38" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N38" s="13" t="n"/>
       <c r="O38" s="13" t="n"/>
-      <c r="P38" s="14" t="inlineStr">
-        <is>
-          <t>1 Jan 2027-1 Sep 2027</t>
-        </is>
+      <c r="P38" s="14" t="n">
+        <v>46416</v>
       </c>
       <c r="Q38" s="17" t="n"/>
       <c r="R38" s="18">
-        <f>IF(AND(P41&lt;&gt;"",Q41&lt;&gt;""),Q41-P41,"")</f>
+        <f>IF(AND(P60&lt;&gt;"",Q60&lt;&gt;""),Q60-P60,"")</f>
         <v/>
       </c>
       <c r="S38" s="13" t="n"/>
       <c r="T38" s="13" t="inlineStr">
         <is>
-          <t>75k-80k</t>
+          <t>66k-75k</t>
         </is>
       </c>
       <c r="U38" s="20" t="inlineStr">
         <is>
-          <t>1-5</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="V38" s="13" t="n"/>
@@ -3894,7 +3914,7 @@
     <row r="39" ht="18" customHeight="1" s="31">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>cisco</t>
+          <t>origin</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
@@ -3904,7 +3924,7 @@
       </c>
       <c r="C39" s="13" t="inlineStr">
         <is>
-          <t>Internship</t>
+          <t>Graduate Program</t>
         </is>
       </c>
       <c r="D39" s="13" t="inlineStr">
@@ -3913,8 +3933,12 @@
         </is>
       </c>
       <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13" t="n"/>
-      <c r="G39" s="13" t="n"/>
+      <c r="F39" s="14" t="n">
+        <v>46166</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>46166</v>
+      </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -3924,13 +3948,17 @@
       <c r="J39" s="13" t="n"/>
       <c r="K39" s="13" t="n"/>
       <c r="L39" s="13" t="n"/>
-      <c r="M39" s="13" t="n"/>
+      <c r="M39" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N39" s="13" t="n"/>
       <c r="O39" s="13" t="n"/>
       <c r="P39" s="13" t="n"/>
       <c r="Q39" s="17" t="n"/>
       <c r="R39" s="18">
-        <f>IF(AND(P43&lt;&gt;"",Q43&lt;&gt;""),Q43-P43,"")</f>
+        <f>IF(AND(P71&lt;&gt;"",Q71&lt;&gt;""),Q71-P71,"")</f>
         <v/>
       </c>
       <c r="S39" s="13" t="n"/>
@@ -3941,55 +3969,74 @@
       <c r="X39" s="13" t="n"/>
       <c r="Y39" s="13" t="n"/>
       <c r="Z39" s="13" t="n"/>
-      <c r="AA39" s="13" t="n"/>
-      <c r="AB39" s="13" t="n"/>
+      <c r="AA39" s="13" t="inlineStr">
+        <is>
+          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
+        </is>
+      </c>
+      <c r="AB39" s="13" t="inlineStr">
+        <is>
+          <t>Customer Churn Forecasting Analysis in Telecom Services, Insurance Risk &amp; Claims Analytics Dashboard, Vendor Performance Analytics Dashboard, Credit Fraud Detection Classifier Analysis</t>
+        </is>
+      </c>
       <c r="AC39" s="13" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="31">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>city of gold coast</t>
+          <t>evolution mining</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>digital and data</t>
+          <t>people and culture</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D40" s="13" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E40" s="13" t="n"/>
       <c r="F40" s="13" t="n"/>
-      <c r="G40" s="13" t="n"/>
+      <c r="G40" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I40" s="13" t="n"/>
-      <c r="J40" s="13" t="n"/>
+      <c r="J40" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K40" s="13" t="n"/>
       <c r="L40" s="13" t="n"/>
       <c r="M40" s="13" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="N40" s="13" t="n"/>
       <c r="O40" s="13" t="n"/>
-      <c r="P40" s="13" t="n"/>
+      <c r="P40" s="14" t="inlineStr">
+        <is>
+          <t>12/1/2026 - 12/31/2026</t>
+        </is>
+      </c>
       <c r="Q40" s="17" t="n"/>
-      <c r="R40" s="18">
-        <f>IF(AND(P44&lt;&gt;"",Q44&lt;&gt;""),Q44-P44,"")</f>
-        <v/>
+      <c r="R40" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S40" s="13" t="n"/>
       <c r="T40" s="13" t="n"/>
@@ -4006,12 +4053,12 @@
     <row r="41" ht="18" customHeight="1" s="31">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>commbank</t>
+          <t>suncorp</t>
         </is>
       </c>
       <c r="B41" s="13" t="inlineStr">
         <is>
-          <t>tech ai engineering data science &amp; ai</t>
+          <t>business analysis non technical</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -4021,41 +4068,52 @@
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="E41" s="13" t="n"/>
       <c r="F41" s="13" t="n"/>
-      <c r="G41" s="13" t="n"/>
+      <c r="G41" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I41" s="13" t="n"/>
-      <c r="J41" s="13" t="n"/>
-      <c r="K41" s="13" t="n"/>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="L41" s="13" t="n"/>
       <c r="M41" s="13" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Rejected</t>
         </is>
       </c>
       <c r="N41" s="13" t="n"/>
       <c r="O41" s="13" t="n"/>
       <c r="P41" s="14" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q41" s="17" t="n"/>
-      <c r="R41" s="18">
-        <f>IF(AND(P45&lt;&gt;"",Q45&lt;&gt;""),Q45-P45,"")</f>
-        <v/>
+        <v>46350</v>
+      </c>
+      <c r="Q41" s="17" t="n">
+        <v>46430</v>
+      </c>
+      <c r="R41" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S41" s="13" t="n"/>
-      <c r="T41" s="13" t="inlineStr">
-        <is>
-          <t>65k</t>
-        </is>
+      <c r="T41" s="13" t="n">
+        <v>37.92</v>
       </c>
       <c r="U41" s="20" t="n"/>
       <c r="V41" s="13" t="n"/>
@@ -4070,52 +4128,69 @@
     <row r="42" ht="18" customHeight="1" s="31">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>eightcap</t>
+          <t>ARUP</t>
         </is>
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>operations analyst</t>
+          <t>digital advisory</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E42" s="13" t="n"/>
       <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
+      <c r="G42" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I42" s="13" t="n"/>
-      <c r="J42" s="13" t="n"/>
+      <c r="J42" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K42" s="13" t="n"/>
       <c r="L42" s="13" t="n"/>
       <c r="M42" s="13" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Applied</t>
         </is>
       </c>
       <c r="N42" s="13" t="n"/>
       <c r="O42" s="13" t="n"/>
-      <c r="P42" s="13" t="n"/>
+      <c r="P42" s="14" t="n">
+        <v>46349</v>
+      </c>
       <c r="Q42" s="17" t="n"/>
-      <c r="R42" s="18">
-        <f>IF(AND(P48&lt;&gt;"",Q48&lt;&gt;""),Q48-P48,"")</f>
-        <v/>
+      <c r="R42" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S42" s="13" t="n"/>
-      <c r="T42" s="13" t="n"/>
-      <c r="U42" s="20" t="n"/>
+      <c r="T42" s="13" t="inlineStr">
+        <is>
+          <t>34-35</t>
+        </is>
+      </c>
+      <c r="U42" s="20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="V42" s="13" t="n"/>
       <c r="W42" s="13" t="n"/>
       <c r="X42" s="13" t="n"/>
@@ -4128,12 +4203,12 @@
     <row r="43" ht="18" customHeight="1" s="31">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>fivecast</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="B43" s="13" t="inlineStr">
         <is>
-          <t>data science</t>
+          <t>data &amp; AI Governance</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -4143,14 +4218,14 @@
       </c>
       <c r="D43" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E43" s="13" t="n"/>
-      <c r="F43" s="14" t="n">
-        <v>46169</v>
-      </c>
-      <c r="G43" s="13" t="n"/>
+      <c r="F43" s="13" t="n"/>
+      <c r="G43" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H43" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4160,14 +4235,21 @@
       <c r="J43" s="13" t="n"/>
       <c r="K43" s="13" t="n"/>
       <c r="L43" s="13" t="n"/>
-      <c r="M43" s="13" t="n"/>
+      <c r="M43" s="13" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
       <c r="N43" s="13" t="n"/>
       <c r="O43" s="13" t="n"/>
-      <c r="P43" s="13" t="n"/>
+      <c r="P43" s="24" t="n">
+        <v>46356</v>
+      </c>
       <c r="Q43" s="17" t="n"/>
-      <c r="R43" s="18">
-        <f>IF(AND(P50&lt;&gt;"",Q50&lt;&gt;""),Q50-P50,"")</f>
-        <v/>
+      <c r="R43" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S43" s="13" t="n"/>
       <c r="T43" s="13" t="n"/>
@@ -4184,48 +4266,71 @@
     <row r="44" ht="18" customHeight="1" s="31">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>flight centre</t>
-        </is>
-      </c>
-      <c r="B44" s="13" t="n"/>
+          <t>Rheinmetall</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr">
+        <is>
+          <t>data analytics</t>
+        </is>
+      </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D44" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E44" s="13" t="n"/>
-      <c r="F44" s="14" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
-      </c>
-      <c r="G44" s="13" t="n"/>
+      <c r="F44" s="13" t="n"/>
+      <c r="G44" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H44" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
       <c r="I44" s="13" t="n"/>
-      <c r="J44" s="13" t="n"/>
+      <c r="J44" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="K44" s="13" t="n"/>
       <c r="L44" s="13" t="n"/>
-      <c r="M44" s="13" t="n"/>
+      <c r="M44" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N44" s="13" t="n"/>
       <c r="O44" s="13" t="n"/>
-      <c r="P44" s="13" t="n"/>
-      <c r="Q44" s="17" t="n"/>
-      <c r="R44" s="18">
-        <f>IF(AND(P51&lt;&gt;"",Q51&lt;&gt;""),Q51-P51,"")</f>
-        <v/>
+      <c r="P44" s="24" t="n">
+        <v>46349</v>
+      </c>
+      <c r="Q44" s="17" t="n">
+        <v>46437</v>
+      </c>
+      <c r="R44" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S44" s="13" t="n"/>
-      <c r="T44" s="13" t="n"/>
-      <c r="U44" s="20" t="n"/>
+      <c r="T44" s="13" t="inlineStr">
+        <is>
+          <t>36 or 66000</t>
+        </is>
+      </c>
+      <c r="U44" s="20" t="inlineStr">
+        <is>
+          <t>5-6</t>
+        </is>
+      </c>
       <c r="V44" s="13" t="n"/>
       <c r="W44" s="13" t="n"/>
       <c r="X44" s="13" t="n"/>
@@ -4238,12 +4343,12 @@
     <row r="45" ht="18" customHeight="1" s="31">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>FTI Consulting</t>
+          <t>grant thornton</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>business consulting</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
@@ -4253,14 +4358,14 @@
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>NSW, WA</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E45" s="13" t="n"/>
-      <c r="F45" s="14" t="n">
-        <v>46093</v>
-      </c>
-      <c r="G45" s="13" t="n"/>
+      <c r="F45" s="13" t="n"/>
+      <c r="G45" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4270,28 +4375,31 @@
       <c r="J45" s="13" t="n"/>
       <c r="K45" s="13" t="n"/>
       <c r="L45" s="13" t="n"/>
-      <c r="M45" s="13" t="n"/>
+      <c r="M45" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N45" s="13" t="n"/>
       <c r="O45" s="13" t="n"/>
-      <c r="P45" s="14" t="inlineStr">
-        <is>
-          <t>4 May 2026 - 18 Jul 2026</t>
+      <c r="P45" s="27" t="inlineStr">
+        <is>
+          <t>11/16/2026 - 18 jan 2027</t>
         </is>
       </c>
       <c r="Q45" s="17" t="n"/>
-      <c r="R45" s="18">
-        <f>IF(AND(P52&lt;&gt;"",Q52&lt;&gt;""),Q52-P52,"")</f>
-        <v/>
+      <c r="R45" s="28" t="inlineStr">
+        <is>
+          <t>4-6 weeks</t>
+        </is>
       </c>
       <c r="S45" s="13" t="n"/>
-      <c r="T45" s="13" t="inlineStr">
-        <is>
-          <t>36 / Hour</t>
-        </is>
+      <c r="T45" s="13" t="n">
+        <v>278</v>
       </c>
       <c r="U45" s="20" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>1-10</t>
         </is>
       </c>
       <c r="V45" s="13" t="n"/>
@@ -4304,33 +4412,31 @@
       <c r="AC45" s="13" t="n"/>
     </row>
     <row r="46" ht="17.25" customHeight="1" s="31">
-      <c r="A46" s="21" t="inlineStr">
-        <is>
-          <t>general motors</t>
-        </is>
-      </c>
-      <c r="B46" s="21" t="inlineStr">
-        <is>
-          <t>Service Operations Business</t>
-        </is>
-      </c>
-      <c r="C46" s="21" t="inlineStr">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>nab</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="inlineStr">
+        <is>
+          <t>digital data and ai</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
       <c r="D46" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E46" s="13" t="n"/>
-      <c r="F46" s="23" t="inlineStr">
-        <is>
-          <t>oct</t>
-        </is>
-      </c>
-      <c r="G46" s="13" t="n"/>
+      <c r="F46" s="13" t="n"/>
+      <c r="G46" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4340,18 +4446,33 @@
       <c r="J46" s="13" t="n"/>
       <c r="K46" s="13" t="n"/>
       <c r="L46" s="13" t="n"/>
-      <c r="M46" s="13" t="n"/>
+      <c r="M46" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N46" s="13" t="n"/>
       <c r="O46" s="13" t="n"/>
-      <c r="P46" s="13" t="n"/>
+      <c r="P46" s="24" t="n">
+        <v>46349</v>
+      </c>
       <c r="Q46" s="17" t="n"/>
-      <c r="R46" s="18">
-        <f>IF(AND(P54&lt;&gt;"",Q54&lt;&gt;""),Q54-P54,"")</f>
-        <v/>
+      <c r="R46" s="28" t="inlineStr">
+        <is>
+          <t>8 weeks</t>
+        </is>
       </c>
       <c r="S46" s="13" t="n"/>
-      <c r="T46" s="13" t="n"/>
-      <c r="U46" s="20" t="n"/>
+      <c r="T46" s="13" t="inlineStr">
+        <is>
+          <t>65000-70000</t>
+        </is>
+      </c>
+      <c r="U46" s="20" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
       <c r="V46" s="13" t="n"/>
       <c r="W46" s="13" t="n"/>
       <c r="X46" s="13" t="n"/>
@@ -4364,27 +4485,29 @@
     <row r="47" ht="18" customHeight="1" s="31">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>hatch</t>
+          <t>AECOM</t>
         </is>
       </c>
       <c r="B47" s="13" t="inlineStr">
         <is>
-          <t>Analyst - Advisory</t>
+          <t>project management</t>
         </is>
       </c>
       <c r="C47" s="13" t="inlineStr">
         <is>
-          <t>Graduate Program</t>
+          <t>Internship</t>
         </is>
       </c>
       <c r="D47" s="13" t="inlineStr">
         <is>
-          <t>NSW</t>
+          <t>VIC</t>
         </is>
       </c>
       <c r="E47" s="13" t="n"/>
       <c r="F47" s="13" t="n"/>
-      <c r="G47" s="13" t="n"/>
+      <c r="G47" s="14" t="n">
+        <v>46096</v>
+      </c>
       <c r="H47" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4394,18 +4517,31 @@
       <c r="J47" s="13" t="n"/>
       <c r="K47" s="13" t="n"/>
       <c r="L47" s="13" t="n"/>
-      <c r="M47" s="13" t="n"/>
+      <c r="M47" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N47" s="13" t="n"/>
       <c r="O47" s="13" t="n"/>
-      <c r="P47" s="13" t="n"/>
+      <c r="P47" s="24" t="n">
+        <v>46342</v>
+      </c>
       <c r="Q47" s="17" t="n"/>
-      <c r="R47" s="18">
-        <f>IF(AND(P55&lt;&gt;"",Q55&lt;&gt;""),Q55-P55,"")</f>
-        <v/>
+      <c r="R47" s="28" t="inlineStr">
+        <is>
+          <t>12 weeks</t>
+        </is>
       </c>
       <c r="S47" s="13" t="n"/>
-      <c r="T47" s="13" t="n"/>
-      <c r="U47" s="20" t="n"/>
+      <c r="T47" s="13" t="n">
+        <v>38</v>
+      </c>
+      <c r="U47" s="20" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
       <c r="V47" s="13" t="n"/>
       <c r="W47" s="13" t="n"/>
       <c r="X47" s="13" t="n"/>
@@ -4418,12 +4554,12 @@
     <row r="48" ht="18" customHeight="1" s="31">
       <c r="A48" s="13" t="inlineStr">
         <is>
-          <t>Heidi Health</t>
+          <t>Commonwealth Bank</t>
         </is>
       </c>
       <c r="B48" s="13" t="inlineStr">
         <is>
-          <t>Strategy &amp; Data Intern</t>
+          <t>Technology &amp; AI -advanced Analytics</t>
         </is>
       </c>
       <c r="C48" s="13" t="inlineStr">
@@ -4433,12 +4569,16 @@
       </c>
       <c r="D48" s="13" t="inlineStr">
         <is>
-          <t>VIC</t>
+          <t>NSW</t>
         </is>
       </c>
       <c r="E48" s="13" t="n"/>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="13" t="n"/>
+      <c r="F48" s="24" t="n">
+        <v>46273</v>
+      </c>
+      <c r="G48" s="29" t="n">
+        <v>46272</v>
+      </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
@@ -4448,20 +4588,31 @@
       <c r="J48" s="13" t="n"/>
       <c r="K48" s="13" t="n"/>
       <c r="L48" s="13" t="n"/>
-      <c r="M48" s="13" t="n"/>
+      <c r="M48" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
       <c r="N48" s="13" t="n"/>
       <c r="O48" s="13" t="n"/>
-      <c r="P48" s="14" t="n">
-        <v>46124</v>
-      </c>
-      <c r="Q48" s="17" t="n"/>
-      <c r="R48" s="18">
-        <f>IF(AND(P56&lt;&gt;"",Q56&lt;&gt;""),Q56-P56,"")</f>
-        <v/>
+      <c r="P48" s="24" t="n">
+        <v>46349</v>
+      </c>
+      <c r="Q48" s="13" t="n"/>
+      <c r="R48" s="28" t="inlineStr">
+        <is>
+          <t>10 weeks</t>
+        </is>
       </c>
       <c r="S48" s="13" t="n"/>
-      <c r="T48" s="13" t="n"/>
-      <c r="U48" s="20" t="n"/>
+      <c r="T48" s="26" t="n">
+        <v>65000</v>
+      </c>
+      <c r="U48" s="20" t="inlineStr">
+        <is>
+          <t>1-8</t>
+        </is>
+      </c>
       <c r="V48" s="13" t="n"/>
       <c r="W48" s="13" t="n"/>
       <c r="X48" s="13" t="n"/>
@@ -4472,2342 +4623,305 @@
       <c r="AC48" s="13" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="31">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>IMC</t>
-        </is>
-      </c>
-      <c r="B49" s="13" t="inlineStr">
-        <is>
-          <t>quantitative research</t>
-        </is>
-      </c>
-      <c r="C49" s="13" t="inlineStr">
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>accenture</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="inlineStr">
+        <is>
+          <t>graduate analyst technology</t>
+        </is>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
+        </is>
+      </c>
+      <c r="D49" s="32" t="inlineStr">
+        <is>
+          <t>VIC</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>46264</v>
+      </c>
+      <c r="H49" s="32" t="inlineStr">
+        <is>
+          <t>Prosple</t>
+        </is>
+      </c>
+      <c r="M49" s="32" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
+        </is>
+      </c>
+      <c r="P49" s="6" t="inlineStr">
+        <is>
+          <t>1/19/2027 - 7/13/2027</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>70000-80000</t>
+        </is>
+      </c>
+      <c r="U49" s="7" t="inlineStr">
+        <is>
+          <t>1-45</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="31">
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t>tiktok</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>business data analyst project intern (GBS)</t>
+        </is>
+      </c>
+      <c r="C50" s="32" t="inlineStr">
         <is>
           <t>Internship</t>
         </is>
       </c>
-      <c r="D49" s="13" t="inlineStr">
+      <c r="D50" s="32" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="E49" s="13" t="n"/>
-      <c r="F49" s="14" t="n">
-        <v>46203</v>
-      </c>
-      <c r="G49" s="13" t="n"/>
-      <c r="H49" s="13" t="inlineStr">
+      <c r="F50" s="6" t="n">
+        <v>46387</v>
+      </c>
+      <c r="G50" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
         <is>
           <t>Prosple</t>
         </is>
       </c>
-      <c r="I49" s="13" t="n"/>
-      <c r="J49" s="13" t="n"/>
-      <c r="K49" s="13" t="n"/>
-      <c r="L49" s="13" t="n"/>
-      <c r="M49" s="13" t="n"/>
-      <c r="N49" s="13" t="n"/>
-      <c r="O49" s="13" t="n"/>
-      <c r="P49" s="13" t="n"/>
-      <c r="Q49" s="17" t="n"/>
-      <c r="R49" s="18">
-        <f>IF(AND(P57&lt;&gt;"",Q57&lt;&gt;""),Q57-P57,"")</f>
-        <v/>
-      </c>
-      <c r="S49" s="13" t="n"/>
-      <c r="T49" s="13" t="n"/>
-      <c r="U49" s="20" t="n"/>
-      <c r="V49" s="13" t="n"/>
-      <c r="W49" s="13" t="n"/>
-      <c r="X49" s="13" t="n"/>
-      <c r="Y49" s="13" t="n"/>
-      <c r="Z49" s="13" t="n"/>
-      <c r="AA49" s="13" t="n"/>
-      <c r="AB49" s="13" t="n"/>
-      <c r="AC49" s="13" t="n"/>
-    </row>
-    <row r="50" ht="15.75" customHeight="1" s="31">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>jpmorganchase</t>
-        </is>
-      </c>
-      <c r="B50" s="13" t="inlineStr">
-        <is>
-          <t>coporate analyst</t>
-        </is>
-      </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
+      <c r="M50" s="32" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>2000-5000 per month</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="31">
+      <c r="A51" s="32" t="inlineStr">
+        <is>
+          <t>Didi</t>
+        </is>
+      </c>
+      <c r="B51" s="32" t="inlineStr">
+        <is>
+          <t>operations intern</t>
+        </is>
+      </c>
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D51" s="32" t="inlineStr">
         <is>
           <t>NSW</t>
         </is>
       </c>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="14" t="n">
-        <v>46108</v>
-      </c>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="13" t="n"/>
-      <c r="K50" s="13" t="n"/>
-      <c r="L50" s="13" t="n"/>
-      <c r="M50" s="13" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="13" t="n"/>
-      <c r="P50" s="13" t="n"/>
-      <c r="Q50" s="17" t="n"/>
-      <c r="R50" s="18">
-        <f>IF(AND(P58&lt;&gt;"",Q58&lt;&gt;""),Q58-P58,"")</f>
-        <v/>
-      </c>
-      <c r="S50" s="13" t="n"/>
-      <c r="T50" s="13" t="n"/>
-      <c r="U50" s="20" t="n"/>
-      <c r="V50" s="13" t="n"/>
-      <c r="W50" s="13" t="n"/>
-      <c r="X50" s="13" t="n"/>
-      <c r="Y50" s="13" t="n"/>
-      <c r="Z50" s="13" t="n"/>
-      <c r="AA50" s="13" t="n"/>
-      <c r="AB50" s="13" t="n"/>
-      <c r="AC50" s="13" t="n"/>
-    </row>
-    <row r="51" ht="15.75" customHeight="1" s="31">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>KPMG</t>
-        </is>
-      </c>
-      <c r="B51" s="13" t="inlineStr">
-        <is>
-          <t>Forensic Risk - Consulting</t>
-        </is>
-      </c>
-      <c r="C51" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="14" t="n">
-        <v>46091</v>
-      </c>
-      <c r="G51" s="13" t="n"/>
-      <c r="H51" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I51" s="13" t="n"/>
-      <c r="J51" s="13" t="n"/>
-      <c r="K51" s="13" t="n"/>
-      <c r="L51" s="13" t="n"/>
-      <c r="M51" s="13" t="n"/>
-      <c r="N51" s="13" t="n"/>
-      <c r="O51" s="13" t="n"/>
-      <c r="P51" s="14" t="n">
-        <v>46426</v>
-      </c>
-      <c r="Q51" s="17" t="n"/>
-      <c r="R51" s="18">
-        <f>IF(AND(P59&lt;&gt;"",Q59&lt;&gt;""),Q59-P59,"")</f>
-        <v/>
-      </c>
-      <c r="S51" s="13" t="n"/>
-      <c r="T51" s="13" t="inlineStr">
-        <is>
-          <t>60k-82k</t>
-        </is>
-      </c>
-      <c r="U51" s="20" t="inlineStr">
-        <is>
-          <t>1-700</t>
-        </is>
-      </c>
-      <c r="V51" s="13" t="n"/>
-      <c r="W51" s="13" t="n"/>
-      <c r="X51" s="13" t="n"/>
-      <c r="Y51" s="13" t="n"/>
-      <c r="Z51" s="13" t="n"/>
-      <c r="AA51" s="13" t="n"/>
-      <c r="AB51" s="13" t="n"/>
-      <c r="AC51" s="13" t="n"/>
+      <c r="G51" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M51" s="32" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="31">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>loreal</t>
-        </is>
-      </c>
-      <c r="B52" s="13" t="inlineStr">
-        <is>
-          <t>Management Trainee Program – Data &amp; Analytics Stream</t>
-        </is>
-      </c>
-      <c r="C52" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="inlineStr">
+      <c r="A52" s="32" t="inlineStr">
+        <is>
+          <t>tencent</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Game Reaserch Development intern, engine reasearch</t>
+        </is>
+      </c>
+      <c r="C52" s="32" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D52" s="32" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="G52" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M52" s="32" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="31">
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>apple</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>information systems and technology</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D53" s="32" t="inlineStr">
+        <is>
+          <t>NSW</t>
+        </is>
+      </c>
+      <c r="G53" s="34" t="n">
+        <v>46277</v>
+      </c>
+      <c r="M53" s="32" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="31">
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>student training and totation program intern</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D54" s="32" t="inlineStr">
         <is>
           <t>VIC</t>
         </is>
       </c>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="14" t="n">
-        <v>46093</v>
-      </c>
-      <c r="G52" s="33" t="n">
+      <c r="G54" s="34" t="n">
         <v>46277</v>
       </c>
-      <c r="H52" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I52" s="13" t="n"/>
-      <c r="J52" s="13" t="n"/>
-      <c r="K52" s="13" t="n"/>
-      <c r="L52" s="13" t="n"/>
-      <c r="M52" s="13" t="inlineStr">
+      <c r="M54" s="32" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="31">
+      <c r="A55" s="32" t="inlineStr">
+        <is>
+          <t>FDM</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Role not recorded</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="G55" s="34" t="n"/>
+      <c r="M55" s="32" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1" s="31">
+      <c r="A56" s="32" t="inlineStr">
+        <is>
+          <t>ADN</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>AusDN Internship Program (Summer 2026/27)</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>Internship</t>
+        </is>
+      </c>
+      <c r="D56" s="32" t="n"/>
+      <c r="G56" s="34" t="n">
+        <v>46281</v>
+      </c>
+      <c r="M56" s="32" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="N52" s="13" t="n"/>
-      <c r="O52" s="13" t="n"/>
-      <c r="P52" s="14" t="n">
-        <v>46416</v>
-      </c>
-      <c r="Q52" s="17" t="n"/>
-      <c r="R52" s="18">
-        <f>IF(AND(P60&lt;&gt;"",Q60&lt;&gt;""),Q60-P60,"")</f>
-        <v/>
-      </c>
-      <c r="S52" s="13" t="n"/>
-      <c r="T52" s="13" t="inlineStr">
-        <is>
-          <t>66k-75k</t>
-        </is>
-      </c>
-      <c r="U52" s="20" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="V52" s="13" t="n"/>
-      <c r="W52" s="13" t="n"/>
-      <c r="X52" s="13" t="n"/>
-      <c r="Y52" s="13" t="n"/>
-      <c r="Z52" s="13" t="n"/>
-      <c r="AA52" s="13" t="n"/>
-      <c r="AB52" s="13" t="n"/>
-      <c r="AC52" s="13" t="n"/>
-    </row>
-    <row r="53" ht="15.75" customHeight="1" s="31">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>McGrathNicol</t>
-        </is>
-      </c>
-      <c r="B53" s="13" t="inlineStr">
-        <is>
-          <t>Data Analytics</t>
-        </is>
-      </c>
-      <c r="C53" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="G53" s="13" t="n"/>
-      <c r="H53" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I53" s="13" t="n"/>
-      <c r="J53" s="13" t="n"/>
-      <c r="K53" s="13" t="n"/>
-      <c r="L53" s="13" t="n"/>
-      <c r="M53" s="13" t="n"/>
-      <c r="N53" s="13" t="n"/>
-      <c r="O53" s="13" t="n"/>
-      <c r="P53" s="14" t="n">
-        <v>46440</v>
-      </c>
-      <c r="Q53" s="17" t="n"/>
-      <c r="R53" s="18">
-        <f>IF(AND(P61&lt;&gt;"",Q61&lt;&gt;""),Q61-P61,"")</f>
-        <v/>
-      </c>
-      <c r="S53" s="13" t="n"/>
-      <c r="T53" s="13" t="inlineStr">
-        <is>
-          <t>78k</t>
-        </is>
-      </c>
-      <c r="U53" s="20" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="V53" s="13" t="n"/>
-      <c r="W53" s="13" t="n"/>
-      <c r="X53" s="13" t="n"/>
-      <c r="Y53" s="13" t="n"/>
-      <c r="Z53" s="13" t="n"/>
-      <c r="AA53" s="13" t="n"/>
-      <c r="AB53" s="13" t="n"/>
-      <c r="AC53" s="13" t="n"/>
-    </row>
-    <row r="54" ht="15.75" customHeight="1" s="31">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>mercedes benz</t>
-        </is>
-      </c>
-      <c r="B54" s="13" t="inlineStr">
-        <is>
-          <t>performance &amp; Insights</t>
-        </is>
-      </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E54" s="13" t="n"/>
-      <c r="F54" s="14" t="inlineStr">
-        <is>
-          <t>oct</t>
-        </is>
-      </c>
-      <c r="G54" s="13" t="n"/>
-      <c r="H54" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I54" s="13" t="n"/>
-      <c r="J54" s="13" t="n"/>
-      <c r="K54" s="13" t="n"/>
-      <c r="L54" s="13" t="n"/>
-      <c r="M54" s="13" t="n"/>
-      <c r="N54" s="13" t="n"/>
-      <c r="O54" s="13" t="n"/>
-      <c r="P54" s="13" t="n"/>
-      <c r="Q54" s="17" t="n"/>
-      <c r="R54" s="18">
-        <f>IF(AND(P63&lt;&gt;"",Q63&lt;&gt;""),Q63-P63,"")</f>
-        <v/>
-      </c>
-      <c r="S54" s="13" t="n"/>
-      <c r="T54" s="13" t="n"/>
-      <c r="U54" s="20" t="n"/>
-      <c r="V54" s="13" t="n"/>
-      <c r="W54" s="13" t="n"/>
-      <c r="X54" s="13" t="n"/>
-      <c r="Y54" s="13" t="n"/>
-      <c r="Z54" s="13" t="n"/>
-      <c r="AA54" s="13" t="n"/>
-      <c r="AB54" s="13" t="n"/>
-      <c r="AC54" s="13" t="n"/>
-    </row>
-    <row r="55" ht="15.75" customHeight="1" s="31">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>moody's corporation</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="inlineStr">
-        <is>
-          <t>Predictive Analytics Intern</t>
-        </is>
-      </c>
-      <c r="C55" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D55" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E55" s="13" t="n"/>
-      <c r="F55" s="14" t="n">
-        <v>46140</v>
-      </c>
-      <c r="G55" s="13" t="n"/>
-      <c r="H55" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I55" s="13" t="n"/>
-      <c r="J55" s="13" t="n"/>
-      <c r="K55" s="13" t="n"/>
-      <c r="L55" s="13" t="n"/>
-      <c r="M55" s="13" t="n"/>
-      <c r="N55" s="13" t="n"/>
-      <c r="O55" s="13" t="n"/>
-      <c r="P55" s="13" t="n"/>
-      <c r="Q55" s="17" t="n"/>
-      <c r="R55" s="18">
-        <f>IF(AND(P64&lt;&gt;"",Q64&lt;&gt;""),Q64-P64,"")</f>
-        <v/>
-      </c>
-      <c r="S55" s="13" t="n"/>
-      <c r="T55" s="13" t="n"/>
-      <c r="U55" s="20" t="n"/>
-      <c r="V55" s="13" t="n"/>
-      <c r="W55" s="13" t="n"/>
-      <c r="X55" s="13" t="n"/>
-      <c r="Y55" s="13" t="n"/>
-      <c r="Z55" s="13" t="n"/>
-      <c r="AA55" s="13" t="n"/>
-      <c r="AB55" s="13" t="n"/>
-      <c r="AC55" s="13" t="n"/>
-    </row>
-    <row r="56" ht="15.75" customHeight="1" s="31">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>nab</t>
-        </is>
-      </c>
-      <c r="B56" s="13" t="inlineStr">
-        <is>
-          <t>digital data and ai</t>
-        </is>
-      </c>
-      <c r="C56" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D56" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E56" s="13" t="n"/>
-      <c r="F56" s="14" t="n">
-        <v>46243</v>
-      </c>
-      <c r="G56" s="13" t="n"/>
-      <c r="H56" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I56" s="13" t="n"/>
-      <c r="J56" s="13" t="n"/>
-      <c r="K56" s="13" t="n"/>
-      <c r="L56" s="13" t="n"/>
-      <c r="M56" s="13" t="n"/>
-      <c r="N56" s="13" t="n"/>
-      <c r="O56" s="13" t="n"/>
-      <c r="P56" s="14" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q56" s="17" t="n"/>
-      <c r="R56" s="18">
-        <f>IF(AND(P65&lt;&gt;"",Q65&lt;&gt;""),Q65-P65,"")</f>
-        <v/>
-      </c>
-      <c r="S56" s="13" t="n"/>
-      <c r="T56" s="13" t="inlineStr">
-        <is>
-          <t>65-70k</t>
-        </is>
-      </c>
-      <c r="U56" s="20" t="n"/>
-      <c r="V56" s="13" t="n"/>
-      <c r="W56" s="13" t="n"/>
-      <c r="X56" s="13" t="n"/>
-      <c r="Y56" s="13" t="n"/>
-      <c r="Z56" s="13" t="n"/>
-      <c r="AA56" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB56" s="13" t="inlineStr">
-        <is>
-          <t>Insurance Risk &amp; Claims Analytics Dashboard, Bank Loan Application Tracking Dashboard, Credit Fraud Detection Classifier Analysis, Customer Segmentation in Bank Campaigns Presentation</t>
-        </is>
-      </c>
-      <c r="AC56" s="13" t="n"/>
-    </row>
-    <row r="57" ht="15.75" customHeight="1" s="31">
-      <c r="A57" s="13" t="inlineStr">
-        <is>
-          <t>nestle</t>
-        </is>
-      </c>
-      <c r="B57" s="13" t="n"/>
-      <c r="C57" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D57" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E57" s="13" t="n"/>
-      <c r="F57" s="14" t="inlineStr">
-        <is>
-          <t>june</t>
-        </is>
-      </c>
-      <c r="G57" s="13" t="n"/>
-      <c r="H57" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I57" s="13" t="n"/>
-      <c r="J57" s="13" t="n"/>
-      <c r="K57" s="13" t="n"/>
-      <c r="L57" s="13" t="n"/>
-      <c r="M57" s="13" t="n"/>
-      <c r="N57" s="13" t="n"/>
-      <c r="O57" s="13" t="n"/>
-      <c r="P57" s="13" t="n"/>
-      <c r="Q57" s="17" t="n"/>
-      <c r="R57" s="18">
-        <f>IF(AND(P66&lt;&gt;"",Q66&lt;&gt;""),Q66-P66,"")</f>
-        <v/>
-      </c>
-      <c r="S57" s="13" t="n"/>
-      <c r="T57" s="13" t="n"/>
-      <c r="U57" s="20" t="n"/>
-      <c r="V57" s="13" t="n"/>
-      <c r="W57" s="13" t="n"/>
-      <c r="X57" s="13" t="n"/>
-      <c r="Y57" s="13" t="n"/>
-      <c r="Z57" s="13" t="n"/>
-      <c r="AA57" s="13" t="n"/>
-      <c r="AB57" s="13" t="n"/>
-      <c r="AC57" s="13" t="n"/>
-    </row>
-    <row r="58" ht="15.75" customHeight="1" s="31">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>NSW government</t>
-        </is>
-      </c>
-      <c r="B58" s="13" t="inlineStr">
-        <is>
-          <t>Data analytics</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D58" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="13" t="n"/>
-      <c r="H58" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I58" s="13" t="n"/>
-      <c r="J58" s="13" t="n"/>
-      <c r="K58" s="13" t="n"/>
-      <c r="L58" s="13" t="n"/>
-      <c r="M58" s="13" t="n"/>
-      <c r="N58" s="13" t="n"/>
-      <c r="O58" s="13" t="n"/>
-      <c r="P58" s="13" t="n"/>
-      <c r="Q58" s="17" t="n"/>
-      <c r="R58" s="18">
-        <f>IF(AND(P67&lt;&gt;"",Q67&lt;&gt;""),Q67-P67,"")</f>
-        <v/>
-      </c>
-      <c r="S58" s="13" t="n"/>
-      <c r="T58" s="13" t="n"/>
-      <c r="U58" s="20" t="n"/>
-      <c r="V58" s="13" t="n"/>
-      <c r="W58" s="13" t="n"/>
-      <c r="X58" s="13" t="n"/>
-      <c r="Y58" s="13" t="n"/>
-      <c r="Z58" s="13" t="n"/>
-      <c r="AA58" s="13" t="n"/>
-      <c r="AB58" s="13" t="n"/>
-      <c r="AC58" s="13" t="n"/>
-    </row>
-    <row r="59" ht="15.75" customHeight="1" s="31">
-      <c r="A59" s="13" t="inlineStr">
-        <is>
-          <t>nti</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Graduate Business Analyst - IT </t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D59" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="14" t="inlineStr">
-        <is>
-          <t>jun</t>
-        </is>
-      </c>
-      <c r="G59" s="13" t="n"/>
-      <c r="H59" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I59" s="13" t="n"/>
-      <c r="J59" s="13" t="n"/>
-      <c r="K59" s="13" t="n"/>
-      <c r="L59" s="13" t="n"/>
-      <c r="M59" s="13" t="n"/>
-      <c r="N59" s="13" t="n"/>
-      <c r="O59" s="13" t="n"/>
-      <c r="P59" s="13" t="n"/>
-      <c r="Q59" s="17" t="n"/>
-      <c r="R59" s="18">
-        <f>IF(AND(P68&lt;&gt;"",Q68&lt;&gt;""),Q68-P68,"")</f>
-        <v/>
-      </c>
-      <c r="S59" s="13" t="n"/>
-      <c r="T59" s="13" t="n"/>
-      <c r="U59" s="20" t="n"/>
-      <c r="V59" s="13" t="n"/>
-      <c r="W59" s="13" t="n"/>
-      <c r="X59" s="13" t="n"/>
-      <c r="Y59" s="13" t="n"/>
-      <c r="Z59" s="13" t="n"/>
-      <c r="AA59" s="13" t="n"/>
-      <c r="AB59" s="13" t="n"/>
-      <c r="AC59" s="13" t="n"/>
-    </row>
-    <row r="60" ht="15.75" customHeight="1" s="31">
-      <c r="A60" s="13" t="inlineStr">
-        <is>
-          <t>optiver</t>
-        </is>
-      </c>
-      <c r="B60" s="13" t="inlineStr">
-        <is>
-          <t>quantitative research</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D60" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="14" t="n">
-        <v>46122</v>
-      </c>
-      <c r="G60" s="13" t="n"/>
-      <c r="H60" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I60" s="13" t="n"/>
-      <c r="J60" s="13" t="n"/>
-      <c r="K60" s="13" t="n"/>
-      <c r="L60" s="13" t="n"/>
-      <c r="M60" s="13" t="n"/>
-      <c r="N60" s="13" t="n"/>
-      <c r="O60" s="13" t="n"/>
-      <c r="P60" s="13" t="n"/>
-      <c r="Q60" s="17" t="n"/>
-      <c r="R60" s="18">
-        <f>IF(AND(P70&lt;&gt;"",Q70&lt;&gt;""),Q70-P70,"")</f>
-        <v/>
-      </c>
-      <c r="S60" s="13" t="n"/>
-      <c r="T60" s="13" t="n"/>
-      <c r="U60" s="20" t="n"/>
-      <c r="V60" s="13" t="n"/>
-      <c r="W60" s="13" t="n"/>
-      <c r="X60" s="13" t="n"/>
-      <c r="Y60" s="13" t="n"/>
-      <c r="Z60" s="13" t="n"/>
-      <c r="AA60" s="13" t="n"/>
-      <c r="AB60" s="13" t="n"/>
-      <c r="AC60" s="13" t="n"/>
-    </row>
-    <row r="61" ht="15.75" customHeight="1" s="31">
-      <c r="A61" s="13" t="inlineStr">
-        <is>
-          <t>origin</t>
-        </is>
-      </c>
-      <c r="B61" s="13" t="inlineStr">
-        <is>
-          <t>business analyst</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D61" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E61" s="13" t="n"/>
-      <c r="F61" s="14" t="n">
-        <v>46166</v>
-      </c>
-      <c r="G61" s="14" t="n">
-        <v>46166</v>
-      </c>
-      <c r="H61" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I61" s="13" t="n"/>
-      <c r="J61" s="13" t="n"/>
-      <c r="K61" s="13" t="n"/>
-      <c r="L61" s="13" t="n"/>
-      <c r="M61" s="13" t="n"/>
-      <c r="N61" s="13" t="n"/>
-      <c r="O61" s="13" t="n"/>
-      <c r="P61" s="13" t="n"/>
-      <c r="Q61" s="17" t="n"/>
-      <c r="R61" s="18">
-        <f>IF(AND(P71&lt;&gt;"",Q71&lt;&gt;""),Q71-P71,"")</f>
-        <v/>
-      </c>
-      <c r="S61" s="13" t="n"/>
-      <c r="T61" s="13" t="n"/>
-      <c r="U61" s="20" t="n"/>
-      <c r="V61" s="13" t="n"/>
-      <c r="W61" s="13" t="n"/>
-      <c r="X61" s="13" t="n"/>
-      <c r="Y61" s="13" t="n"/>
-      <c r="Z61" s="13" t="n"/>
-      <c r="AA61" s="13" t="inlineStr">
-        <is>
-          <t>NDIS Quality and Safeguards Commission Data Analyst Intern</t>
-        </is>
-      </c>
-      <c r="AB61" s="13" t="inlineStr">
-        <is>
-          <t>Customer Churn Forecasting Analysis in Telecom Services, Insurance Risk &amp; Claims Analytics Dashboard, Vendor Performance Analytics Dashboard, Credit Fraud Detection Classifier Analysis</t>
-        </is>
-      </c>
-      <c r="AC61" s="13" t="n"/>
-    </row>
-    <row r="62" ht="15.75" customHeight="1" s="31">
-      <c r="A62" s="13" t="inlineStr">
-        <is>
-          <t>QBE Insurance</t>
-        </is>
-      </c>
-      <c r="B62" s="13" t="inlineStr">
-        <is>
-          <t>data analytics</t>
-        </is>
-      </c>
-      <c r="C62" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D62" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E62" s="13" t="n"/>
-      <c r="F62" s="14" t="n">
-        <v>46253</v>
-      </c>
-      <c r="G62" s="13" t="n"/>
-      <c r="H62" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I62" s="13" t="n"/>
-      <c r="J62" s="13" t="n"/>
-      <c r="K62" s="13" t="n"/>
-      <c r="L62" s="13" t="n"/>
-      <c r="M62" s="13" t="n"/>
-      <c r="N62" s="13" t="n"/>
-      <c r="O62" s="13" t="n"/>
-      <c r="P62" s="13" t="n"/>
-      <c r="Q62" s="17" t="n"/>
-      <c r="R62" s="18">
-        <f>IF(AND(P72&lt;&gt;"",Q72&lt;&gt;""),Q72-P72,"")</f>
-        <v/>
-      </c>
-      <c r="S62" s="13" t="n"/>
-      <c r="T62" s="13" t="n"/>
-      <c r="U62" s="20" t="n"/>
-      <c r="V62" s="13" t="n"/>
-      <c r="W62" s="13" t="n"/>
-      <c r="X62" s="13" t="n"/>
-      <c r="Y62" s="13" t="n"/>
-      <c r="Z62" s="13" t="n"/>
-      <c r="AA62" s="13" t="n"/>
-      <c r="AB62" s="13" t="n"/>
-      <c r="AC62" s="13" t="n"/>
-    </row>
-    <row r="63" ht="15.75" customHeight="1" s="31">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">queensland government digital </t>
-        </is>
-      </c>
-      <c r="B63" s="13" t="inlineStr">
-        <is>
-          <t>Data analytics</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>Graduate School</t>
-        </is>
-      </c>
-      <c r="D63" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="13" t="n"/>
-      <c r="G63" s="13" t="n"/>
-      <c r="H63" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I63" s="13" t="n"/>
-      <c r="J63" s="13" t="n"/>
-      <c r="K63" s="13" t="n"/>
-      <c r="L63" s="13" t="n"/>
-      <c r="M63" s="13" t="n"/>
-      <c r="N63" s="13" t="n"/>
-      <c r="O63" s="13" t="n"/>
-      <c r="P63" s="13" t="n"/>
-      <c r="Q63" s="17" t="n"/>
-      <c r="R63" s="18">
-        <f>IF(AND(P73&lt;&gt;"",Q73&lt;&gt;""),Q73-P73,"")</f>
-        <v/>
-      </c>
-      <c r="S63" s="13" t="n"/>
-      <c r="T63" s="13" t="n"/>
-      <c r="U63" s="20" t="n"/>
-      <c r="V63" s="13" t="n"/>
-      <c r="W63" s="13" t="n"/>
-      <c r="X63" s="13" t="n"/>
-      <c r="Y63" s="13" t="n"/>
-      <c r="Z63" s="13" t="n"/>
-      <c r="AA63" s="13" t="n"/>
-      <c r="AB63" s="13" t="n"/>
-      <c r="AC63" s="13" t="n"/>
-    </row>
-    <row r="64" ht="15.75" customHeight="1" s="31">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>shell</t>
-        </is>
-      </c>
-      <c r="B64" s="13" t="inlineStr">
-        <is>
-          <t>business analyst</t>
-        </is>
-      </c>
-      <c r="C64" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D64" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="14" t="inlineStr">
-        <is>
-          <t>sep</t>
-        </is>
-      </c>
-      <c r="G64" s="13" t="n"/>
-      <c r="H64" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I64" s="13" t="n"/>
-      <c r="J64" s="13" t="n"/>
-      <c r="K64" s="13" t="n"/>
-      <c r="L64" s="13" t="n"/>
-      <c r="M64" s="13" t="n"/>
-      <c r="N64" s="13" t="n"/>
-      <c r="O64" s="13" t="n"/>
-      <c r="P64" s="13" t="n"/>
-      <c r="Q64" s="17" t="n"/>
-      <c r="R64" s="18">
-        <f>IF(AND(P74&lt;&gt;"",Q74&lt;&gt;""),Q74-P74,"")</f>
-        <v/>
-      </c>
-      <c r="S64" s="13" t="n"/>
-      <c r="T64" s="13" t="n"/>
-      <c r="U64" s="20" t="n"/>
-      <c r="V64" s="13" t="n"/>
-      <c r="W64" s="13" t="n"/>
-      <c r="X64" s="13" t="n"/>
-      <c r="Y64" s="13" t="n"/>
-      <c r="Z64" s="13" t="n"/>
-      <c r="AA64" s="13" t="n"/>
-      <c r="AB64" s="13" t="n"/>
-      <c r="AC64" s="13" t="n"/>
-    </row>
-    <row r="65" ht="15.75" customHeight="1" s="31">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>sportsbet</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Graduate Data Scientist Risk &amp; Pricing </t>
-        </is>
-      </c>
-      <c r="C65" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D65" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E65" s="13" t="n"/>
-      <c r="F65" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="G65" s="13" t="n"/>
-      <c r="H65" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I65" s="13" t="n"/>
-      <c r="J65" s="13" t="n"/>
-      <c r="K65" s="13" t="n"/>
-      <c r="L65" s="13" t="n"/>
-      <c r="M65" s="13" t="n"/>
-      <c r="N65" s="13" t="n"/>
-      <c r="O65" s="13" t="n"/>
-      <c r="P65" s="13" t="n"/>
-      <c r="Q65" s="17" t="n"/>
-      <c r="R65" s="18">
-        <f>IF(AND(P75&lt;&gt;"",Q75&lt;&gt;""),Q75-P75,"")</f>
-        <v/>
-      </c>
-      <c r="S65" s="13" t="n"/>
-      <c r="T65" s="13" t="n"/>
-      <c r="U65" s="20" t="n"/>
-      <c r="V65" s="13" t="n"/>
-      <c r="W65" s="13" t="n"/>
-      <c r="X65" s="13" t="n"/>
-      <c r="Y65" s="13" t="n"/>
-      <c r="Z65" s="13" t="n"/>
-      <c r="AA65" s="13" t="n"/>
-      <c r="AB65" s="13" t="n"/>
-      <c r="AC65" s="13" t="n"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1" s="31">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>streem</t>
-        </is>
-      </c>
-      <c r="B66" s="13" t="inlineStr">
-        <is>
-          <t>Junior Media Analyst - Remote</t>
-        </is>
-      </c>
-      <c r="C66" s="13" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="D66" s="13" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E66" s="13" t="n"/>
-      <c r="F66" s="13" t="n"/>
-      <c r="G66" s="13" t="n"/>
-      <c r="H66" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I66" s="13" t="n"/>
-      <c r="J66" s="13" t="n"/>
-      <c r="K66" s="13" t="n"/>
-      <c r="L66" s="13" t="n"/>
-      <c r="M66" s="13" t="n"/>
-      <c r="N66" s="13" t="n"/>
-      <c r="O66" s="13" t="n"/>
-      <c r="P66" s="13" t="n"/>
-      <c r="Q66" s="17" t="n"/>
-      <c r="R66" s="18">
-        <f>IF(AND(P77&lt;&gt;"",Q77&lt;&gt;""),Q77-P77,"")</f>
-        <v/>
-      </c>
-      <c r="S66" s="13" t="n"/>
-      <c r="T66" s="13" t="n"/>
-      <c r="U66" s="20" t="n"/>
-      <c r="V66" s="13" t="n"/>
-      <c r="W66" s="13" t="n"/>
-      <c r="X66" s="13" t="n"/>
-      <c r="Y66" s="13" t="n"/>
-      <c r="Z66" s="13" t="n"/>
-      <c r="AA66" s="13" t="n"/>
-      <c r="AB66" s="13" t="n"/>
-      <c r="AC66" s="13" t="n"/>
-    </row>
-    <row r="67" ht="15.75" customHeight="1" s="31">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>suncorp</t>
-        </is>
-      </c>
-      <c r="B67" s="13" t="n"/>
-      <c r="C67" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D67" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="14" t="inlineStr">
-        <is>
-          <t>aug</t>
-        </is>
-      </c>
-      <c r="G67" s="13" t="n"/>
-      <c r="H67" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I67" s="13" t="n"/>
-      <c r="J67" s="13" t="n"/>
-      <c r="K67" s="13" t="n"/>
-      <c r="L67" s="13" t="n"/>
-      <c r="M67" s="13" t="n"/>
-      <c r="N67" s="13" t="n"/>
-      <c r="O67" s="13" t="n"/>
-      <c r="P67" s="13" t="n"/>
-      <c r="Q67" s="17" t="n"/>
-      <c r="R67" s="18">
-        <f>IF(AND(P78&lt;&gt;"",Q78&lt;&gt;""),Q78-P78,"")</f>
-        <v/>
-      </c>
-      <c r="S67" s="13" t="n"/>
-      <c r="T67" s="13" t="n"/>
-      <c r="U67" s="20" t="n"/>
-      <c r="V67" s="13" t="n"/>
-      <c r="W67" s="13" t="n"/>
-      <c r="X67" s="13" t="n"/>
-      <c r="Y67" s="13" t="n"/>
-      <c r="Z67" s="13" t="n"/>
-      <c r="AA67" s="13" t="n"/>
-      <c r="AB67" s="13" t="n"/>
-      <c r="AC67" s="13" t="n"/>
-    </row>
-    <row r="68" ht="15.75" customHeight="1" s="31">
-      <c r="A68" s="13" t="inlineStr">
-        <is>
-          <t>ventia</t>
-        </is>
-      </c>
-      <c r="B68" s="13" t="inlineStr">
-        <is>
-          <t>data science &amp; analysics graduate</t>
-        </is>
-      </c>
-      <c r="C68" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D68" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="G68" s="13" t="n"/>
-      <c r="H68" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I68" s="13" t="n"/>
-      <c r="J68" s="13" t="n"/>
-      <c r="K68" s="13" t="n"/>
-      <c r="L68" s="13" t="n"/>
-      <c r="M68" s="13" t="n"/>
-      <c r="N68" s="13" t="n"/>
-      <c r="O68" s="13" t="n"/>
-      <c r="P68" s="14" t="n">
-        <v>46047</v>
-      </c>
-      <c r="Q68" s="17" t="n"/>
-      <c r="R68" s="18">
-        <f>IF(AND(P79&lt;&gt;"",Q79&lt;&gt;""),Q79-P79,"")</f>
-        <v/>
-      </c>
-      <c r="S68" s="13" t="n"/>
-      <c r="T68" s="13" t="inlineStr">
-        <is>
-          <t>70-80k</t>
-        </is>
-      </c>
-      <c r="U68" s="20" t="n"/>
-      <c r="V68" s="13" t="n"/>
-      <c r="W68" s="13" t="n"/>
-      <c r="X68" s="13" t="n"/>
-      <c r="Y68" s="13" t="n"/>
-      <c r="Z68" s="13" t="n"/>
-      <c r="AA68" s="13" t="n"/>
-      <c r="AB68" s="13" t="n"/>
-      <c r="AC68" s="13" t="n"/>
-    </row>
-    <row r="69" ht="15.75" customHeight="1" s="31">
-      <c r="A69" s="13" t="inlineStr">
-        <is>
-          <t>Visa</t>
-        </is>
-      </c>
-      <c r="B69" s="13" t="inlineStr">
-        <is>
-          <t>data science consulting</t>
-        </is>
-      </c>
-      <c r="C69" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D69" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E69" s="13" t="n"/>
-      <c r="F69" s="13" t="n"/>
-      <c r="G69" s="13" t="n"/>
-      <c r="H69" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I69" s="13" t="n"/>
-      <c r="J69" s="13" t="n"/>
-      <c r="K69" s="13" t="n"/>
-      <c r="L69" s="13" t="n"/>
-      <c r="M69" s="13" t="n"/>
-      <c r="N69" s="13" t="n"/>
-      <c r="O69" s="13" t="n"/>
-      <c r="P69" s="13" t="n"/>
-      <c r="Q69" s="17" t="n"/>
-      <c r="R69" s="18">
-        <f>IF(AND(P80&lt;&gt;"",Q80&lt;&gt;""),Q80-P80,"")</f>
-        <v/>
-      </c>
-      <c r="S69" s="13" t="n"/>
-      <c r="T69" s="13" t="n"/>
-      <c r="U69" s="20" t="n"/>
-      <c r="V69" s="13" t="n"/>
-      <c r="W69" s="13" t="n"/>
-      <c r="X69" s="13" t="n"/>
-      <c r="Y69" s="13" t="n"/>
-      <c r="Z69" s="13" t="n"/>
-      <c r="AA69" s="13" t="n"/>
-      <c r="AB69" s="13" t="n"/>
-      <c r="AC69" s="13" t="n"/>
-    </row>
-    <row r="70" ht="15.75" customHeight="1" s="31">
-      <c r="A70" s="13" t="inlineStr">
-        <is>
-          <t>visagio</t>
-        </is>
-      </c>
-      <c r="B70" s="13" t="inlineStr">
-        <is>
-          <t>data &amp; analytics consultant</t>
-        </is>
-      </c>
-      <c r="C70" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D70" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E70" s="13" t="n"/>
-      <c r="F70" s="14" t="n">
-        <v>46105</v>
-      </c>
-      <c r="G70" s="13" t="n"/>
-      <c r="H70" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I70" s="13" t="n"/>
-      <c r="J70" s="13" t="n"/>
-      <c r="K70" s="13" t="n"/>
-      <c r="L70" s="13" t="n"/>
-      <c r="M70" s="13" t="n"/>
-      <c r="N70" s="13" t="n"/>
-      <c r="O70" s="13" t="n"/>
-      <c r="P70" s="13" t="n"/>
-      <c r="Q70" s="17" t="n"/>
-      <c r="R70" s="18">
-        <f>IF(AND(P81&lt;&gt;"",Q81&lt;&gt;""),Q81-P81,"")</f>
-        <v/>
-      </c>
-      <c r="S70" s="13" t="n"/>
-      <c r="T70" s="13" t="n"/>
-      <c r="U70" s="20" t="n"/>
-      <c r="V70" s="13" t="n"/>
-      <c r="W70" s="13" t="n"/>
-      <c r="X70" s="13" t="n"/>
-      <c r="Y70" s="13" t="n"/>
-      <c r="Z70" s="13" t="n"/>
-      <c r="AA70" s="13" t="n"/>
-      <c r="AB70" s="13" t="n"/>
-      <c r="AC70" s="13" t="n"/>
-    </row>
-    <row r="71" ht="15.75" customHeight="1" s="31">
-      <c r="A71" s="13" t="inlineStr">
-        <is>
-          <t>Vistar Media</t>
-        </is>
-      </c>
-      <c r="B71" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Analytics Associate </t>
-        </is>
-      </c>
-      <c r="C71" s="13" t="inlineStr">
-        <is>
-          <t>Full-time</t>
-        </is>
-      </c>
-      <c r="D71" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E71" s="13" t="n"/>
-      <c r="F71" s="13" t="n"/>
-      <c r="G71" s="13" t="n"/>
-      <c r="H71" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I71" s="13" t="n"/>
-      <c r="J71" s="13" t="n"/>
-      <c r="K71" s="13" t="n"/>
-      <c r="L71" s="13" t="n"/>
-      <c r="M71" s="13" t="n"/>
-      <c r="N71" s="13" t="n"/>
-      <c r="O71" s="13" t="n"/>
-      <c r="P71" s="13" t="n"/>
-      <c r="Q71" s="17" t="n"/>
-      <c r="R71" s="18">
-        <f>IF(AND(P82&lt;&gt;"",Q82&lt;&gt;""),Q82-P82,"")</f>
-        <v/>
-      </c>
-      <c r="S71" s="13" t="n"/>
-      <c r="T71" s="13" t="n"/>
-      <c r="U71" s="20" t="n"/>
-      <c r="V71" s="13" t="n"/>
-      <c r="W71" s="13" t="n"/>
-      <c r="X71" s="13" t="n"/>
-      <c r="Y71" s="13" t="n"/>
-      <c r="Z71" s="13" t="n"/>
-      <c r="AA71" s="13" t="n"/>
-      <c r="AB71" s="13" t="n"/>
-      <c r="AC71" s="13" t="n"/>
-    </row>
-    <row r="72" ht="15.75" customHeight="1" s="31">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>Westpac</t>
-        </is>
-      </c>
-      <c r="B72" s="13" t="inlineStr">
-        <is>
-          <t>Technology (Data)</t>
-        </is>
-      </c>
-      <c r="C72" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D72" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="G72" s="13" t="n"/>
-      <c r="H72" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I72" s="13" t="n"/>
-      <c r="J72" s="13" t="n"/>
-      <c r="K72" s="13" t="n"/>
-      <c r="L72" s="13" t="n"/>
-      <c r="M72" s="13" t="n"/>
-      <c r="N72" s="13" t="n"/>
-      <c r="O72" s="13" t="n"/>
-      <c r="P72" s="14" t="inlineStr">
-        <is>
-          <t>1 Feb 2027 - 28 Feb 2027</t>
-        </is>
-      </c>
-      <c r="Q72" s="17" t="n"/>
-      <c r="R72" s="18">
-        <f>IF(AND(P83&lt;&gt;"",Q83&lt;&gt;""),Q83-P83,"")</f>
-        <v/>
-      </c>
-      <c r="S72" s="13" t="n"/>
-      <c r="T72" s="13" t="inlineStr">
-        <is>
-          <t>80k-90k</t>
-        </is>
-      </c>
-      <c r="U72" s="20" t="inlineStr">
-        <is>
-          <t>1-100</t>
-        </is>
-      </c>
-      <c r="V72" s="13" t="n"/>
-      <c r="W72" s="13" t="n"/>
-      <c r="X72" s="13" t="n"/>
-      <c r="Y72" s="13" t="n"/>
-      <c r="Z72" s="13" t="n"/>
-      <c r="AA72" s="13" t="n"/>
-      <c r="AB72" s="13" t="n"/>
-      <c r="AC72" s="13" t="n"/>
-    </row>
-    <row r="73" ht="15.75" customHeight="1" s="31">
-      <c r="A73" s="13" t="inlineStr">
-        <is>
-          <t>westpac</t>
-        </is>
-      </c>
-      <c r="B73" s="13" t="inlineStr">
-        <is>
-          <t>data digital ai</t>
-        </is>
-      </c>
-      <c r="C73" s="13" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D73" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E73" s="13" t="n"/>
-      <c r="F73" s="14" t="n">
-        <v>46248</v>
-      </c>
-      <c r="G73" s="13" t="n"/>
-      <c r="H73" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I73" s="13" t="n"/>
-      <c r="J73" s="13" t="n"/>
-      <c r="K73" s="13" t="n"/>
-      <c r="L73" s="13" t="n"/>
-      <c r="M73" s="13" t="n"/>
-      <c r="N73" s="13" t="n"/>
-      <c r="O73" s="13" t="n"/>
-      <c r="P73" s="14" t="n">
-        <v>46068</v>
-      </c>
-      <c r="Q73" s="17" t="n"/>
-      <c r="R73" s="18">
-        <f>IF(AND(P84&lt;&gt;"",Q84&lt;&gt;""),Q84-P84,"")</f>
-        <v/>
-      </c>
-      <c r="S73" s="13" t="n"/>
-      <c r="T73" s="13" t="inlineStr">
-        <is>
-          <t>80-90k</t>
-        </is>
-      </c>
-      <c r="U73" s="20" t="n"/>
-      <c r="V73" s="13" t="n"/>
-      <c r="W73" s="13" t="n"/>
-      <c r="X73" s="13" t="n"/>
-      <c r="Y73" s="13" t="n"/>
-      <c r="Z73" s="13" t="n"/>
-      <c r="AA73" s="13" t="n"/>
-      <c r="AB73" s="13" t="n"/>
-      <c r="AC73" s="13" t="n"/>
-    </row>
-    <row r="74" ht="15.75" customHeight="1" s="31">
-      <c r="A74" s="13" t="inlineStr">
-        <is>
-          <t>evolution mining</t>
-        </is>
-      </c>
-      <c r="B74" s="13" t="inlineStr">
-        <is>
-          <t>people and culture</t>
-        </is>
-      </c>
-      <c r="C74" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D74" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E74" s="13" t="n"/>
-      <c r="F74" s="13" t="n"/>
-      <c r="G74" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H74" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I74" s="13" t="n"/>
-      <c r="J74" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K74" s="13" t="n"/>
-      <c r="L74" s="13" t="n"/>
-      <c r="M74" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N74" s="13" t="n"/>
-      <c r="O74" s="13" t="n"/>
-      <c r="P74" s="14" t="inlineStr">
-        <is>
-          <t>12/1/2026 - 12/31/2026</t>
-        </is>
-      </c>
-      <c r="Q74" s="17" t="n"/>
-      <c r="R74" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S74" s="13" t="n"/>
-      <c r="T74" s="13" t="n"/>
-      <c r="U74" s="20" t="n"/>
-      <c r="V74" s="13" t="n"/>
-      <c r="W74" s="13" t="n"/>
-      <c r="X74" s="13" t="n"/>
-      <c r="Y74" s="13" t="n"/>
-      <c r="Z74" s="13" t="n"/>
-      <c r="AA74" s="13" t="n"/>
-      <c r="AB74" s="13" t="n"/>
-      <c r="AC74" s="13" t="n"/>
-    </row>
-    <row r="75" ht="15.75" customHeight="1" s="31">
-      <c r="A75" s="13" t="inlineStr">
-        <is>
-          <t>suncorp</t>
-        </is>
-      </c>
-      <c r="B75" s="13" t="inlineStr">
-        <is>
-          <t>business analysis non technical</t>
-        </is>
-      </c>
-      <c r="C75" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D75" s="13" t="inlineStr">
-        <is>
-          <t>QLD</t>
-        </is>
-      </c>
-      <c r="E75" s="13" t="n"/>
-      <c r="F75" s="13" t="n"/>
-      <c r="G75" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H75" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I75" s="13" t="n"/>
-      <c r="J75" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K75" s="13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="L75" s="13" t="n"/>
-      <c r="M75" s="13" t="inlineStr">
-        <is>
-          <t>Finished Assessment</t>
-        </is>
-      </c>
-      <c r="N75" s="13" t="n"/>
-      <c r="O75" s="13" t="n"/>
-      <c r="P75" s="14" t="n">
-        <v>46350</v>
-      </c>
-      <c r="Q75" s="17" t="n">
-        <v>46430</v>
-      </c>
-      <c r="R75" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S75" s="13" t="n"/>
-      <c r="T75" s="13" t="n">
-        <v>37.92</v>
-      </c>
-      <c r="U75" s="20" t="n"/>
-      <c r="V75" s="13" t="n"/>
-      <c r="W75" s="13" t="n"/>
-      <c r="X75" s="13" t="n"/>
-      <c r="Y75" s="13" t="n"/>
-      <c r="Z75" s="13" t="n"/>
-      <c r="AA75" s="13" t="n"/>
-      <c r="AB75" s="13" t="n"/>
-      <c r="AC75" s="13" t="n"/>
-    </row>
-    <row r="76" ht="15.75" customHeight="1" s="31">
-      <c r="A76" s="13" t="inlineStr">
-        <is>
-          <t>ARUP</t>
-        </is>
-      </c>
-      <c r="B76" s="13" t="inlineStr">
-        <is>
-          <t>digital advisory</t>
-        </is>
-      </c>
-      <c r="C76" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D76" s="13" t="inlineStr">
-        <is>
-          <t>Hong Kong</t>
-        </is>
-      </c>
-      <c r="E76" s="13" t="n"/>
-      <c r="F76" s="13" t="n"/>
-      <c r="G76" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H76" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I76" s="13" t="n"/>
-      <c r="J76" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K76" s="13" t="n"/>
-      <c r="L76" s="13" t="n"/>
-      <c r="M76" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N76" s="13" t="n"/>
-      <c r="O76" s="13" t="n"/>
-      <c r="P76" s="14" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q76" s="17" t="n"/>
-      <c r="R76" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S76" s="13" t="n"/>
-      <c r="T76" s="13" t="inlineStr">
-        <is>
-          <t>34-35</t>
-        </is>
-      </c>
-      <c r="U76" s="20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="V76" s="13" t="n"/>
-      <c r="W76" s="13" t="n"/>
-      <c r="X76" s="13" t="n"/>
-      <c r="Y76" s="13" t="n"/>
-      <c r="Z76" s="13" t="n"/>
-      <c r="AA76" s="13" t="n"/>
-      <c r="AB76" s="13" t="n"/>
-      <c r="AC76" s="13" t="n"/>
-    </row>
-    <row r="77" ht="15.75" customHeight="1" s="31">
-      <c r="A77" s="13" t="inlineStr">
-        <is>
-          <t>APA</t>
-        </is>
-      </c>
-      <c r="B77" s="13" t="inlineStr">
-        <is>
-          <t>data &amp; AI Governance</t>
-        </is>
-      </c>
-      <c r="C77" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D77" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E77" s="13" t="n"/>
-      <c r="F77" s="13" t="n"/>
-      <c r="G77" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H77" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I77" s="13" t="n"/>
-      <c r="J77" s="13" t="n"/>
-      <c r="K77" s="13" t="n"/>
-      <c r="L77" s="13" t="n"/>
-      <c r="M77" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N77" s="13" t="n"/>
-      <c r="O77" s="13" t="n"/>
-      <c r="P77" s="24" t="n">
-        <v>46356</v>
-      </c>
-      <c r="Q77" s="17" t="n"/>
-      <c r="R77" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S77" s="13" t="n"/>
-      <c r="T77" s="13" t="n"/>
-      <c r="U77" s="20" t="n"/>
-      <c r="V77" s="13" t="n"/>
-      <c r="W77" s="13" t="n"/>
-      <c r="X77" s="13" t="n"/>
-      <c r="Y77" s="13" t="n"/>
-      <c r="Z77" s="13" t="n"/>
-      <c r="AA77" s="13" t="n"/>
-      <c r="AB77" s="13" t="n"/>
-      <c r="AC77" s="13" t="n"/>
-    </row>
-    <row r="78" ht="15.75" customHeight="1" s="31">
-      <c r="A78" s="13" t="inlineStr">
-        <is>
-          <t>Rheinmetall</t>
-        </is>
-      </c>
-      <c r="B78" s="13" t="inlineStr">
-        <is>
-          <t>data analytics</t>
-        </is>
-      </c>
-      <c r="C78" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D78" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n"/>
-      <c r="G78" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H78" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I78" s="13" t="n"/>
-      <c r="J78" s="13" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K78" s="13" t="n"/>
-      <c r="L78" s="13" t="n"/>
-      <c r="M78" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N78" s="13" t="n"/>
-      <c r="O78" s="13" t="n"/>
-      <c r="P78" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q78" s="17" t="n">
-        <v>46437</v>
-      </c>
-      <c r="R78" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S78" s="13" t="n"/>
-      <c r="T78" s="13" t="inlineStr">
-        <is>
-          <t>36 or 66000</t>
-        </is>
-      </c>
-      <c r="U78" s="20" t="inlineStr">
-        <is>
-          <t>5-6</t>
-        </is>
-      </c>
-      <c r="V78" s="13" t="n"/>
-      <c r="W78" s="13" t="n"/>
-      <c r="X78" s="13" t="n"/>
-      <c r="Y78" s="13" t="n"/>
-      <c r="Z78" s="13" t="n"/>
-      <c r="AA78" s="13" t="n"/>
-      <c r="AB78" s="13" t="n"/>
-      <c r="AC78" s="13" t="n"/>
-    </row>
-    <row r="79" ht="15.75" customHeight="1" s="31">
-      <c r="A79" s="13" t="inlineStr">
-        <is>
-          <t>grant thornton</t>
-        </is>
-      </c>
-      <c r="B79" s="13" t="inlineStr">
-        <is>
-          <t>business consulting</t>
-        </is>
-      </c>
-      <c r="C79" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D79" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E79" s="13" t="n"/>
-      <c r="F79" s="13" t="n"/>
-      <c r="G79" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H79" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I79" s="13" t="n"/>
-      <c r="J79" s="13" t="n"/>
-      <c r="K79" s="13" t="n"/>
-      <c r="L79" s="13" t="n"/>
-      <c r="M79" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N79" s="13" t="n"/>
-      <c r="O79" s="13" t="n"/>
-      <c r="P79" s="27" t="inlineStr">
-        <is>
-          <t>11/16/2026 - 18 jan 2027</t>
-        </is>
-      </c>
-      <c r="Q79" s="17" t="n"/>
-      <c r="R79" s="28" t="inlineStr">
-        <is>
-          <t>4-6 weeks</t>
-        </is>
-      </c>
-      <c r="S79" s="13" t="n"/>
-      <c r="T79" s="13" t="n">
-        <v>278</v>
-      </c>
-      <c r="U79" s="20" t="inlineStr">
-        <is>
-          <t>1-10</t>
-        </is>
-      </c>
-      <c r="V79" s="13" t="n"/>
-      <c r="W79" s="13" t="n"/>
-      <c r="X79" s="13" t="n"/>
-      <c r="Y79" s="13" t="n"/>
-      <c r="Z79" s="13" t="n"/>
-      <c r="AA79" s="13" t="n"/>
-      <c r="AB79" s="13" t="n"/>
-      <c r="AC79" s="13" t="n"/>
-    </row>
-    <row r="80" ht="15.75" customHeight="1" s="31">
-      <c r="A80" s="13" t="inlineStr">
-        <is>
-          <t>nab</t>
-        </is>
-      </c>
-      <c r="B80" s="13" t="inlineStr">
-        <is>
-          <t>digital data and ai</t>
-        </is>
-      </c>
-      <c r="C80" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D80" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E80" s="13" t="n"/>
-      <c r="F80" s="13" t="n"/>
-      <c r="G80" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H80" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I80" s="13" t="n"/>
-      <c r="J80" s="13" t="n"/>
-      <c r="K80" s="13" t="n"/>
-      <c r="L80" s="13" t="n"/>
-      <c r="M80" s="13" t="inlineStr">
-        <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="N80" s="13" t="n"/>
-      <c r="O80" s="13" t="n"/>
-      <c r="P80" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q80" s="17" t="n"/>
-      <c r="R80" s="28" t="inlineStr">
-        <is>
-          <t>8 weeks</t>
-        </is>
-      </c>
-      <c r="S80" s="13" t="n"/>
-      <c r="T80" s="13" t="inlineStr">
-        <is>
-          <t>65000-70000</t>
-        </is>
-      </c>
-      <c r="U80" s="20" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="V80" s="13" t="n"/>
-      <c r="W80" s="13" t="n"/>
-      <c r="X80" s="13" t="n"/>
-      <c r="Y80" s="13" t="n"/>
-      <c r="Z80" s="13" t="n"/>
-      <c r="AA80" s="13" t="n"/>
-      <c r="AB80" s="13" t="n"/>
-      <c r="AC80" s="13" t="n"/>
-    </row>
-    <row r="81" ht="15.75" customHeight="1" s="31">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>AECOM</t>
-        </is>
-      </c>
-      <c r="B81" s="13" t="inlineStr">
-        <is>
-          <t>project management</t>
-        </is>
-      </c>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D81" s="13" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="E81" s="13" t="n"/>
-      <c r="F81" s="13" t="n"/>
-      <c r="G81" s="14" t="n">
-        <v>46096</v>
-      </c>
-      <c r="H81" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I81" s="13" t="n"/>
-      <c r="J81" s="13" t="n"/>
-      <c r="K81" s="13" t="n"/>
-      <c r="L81" s="13" t="n"/>
-      <c r="M81" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N81" s="13" t="n"/>
-      <c r="O81" s="13" t="n"/>
-      <c r="P81" s="24" t="n">
-        <v>46342</v>
-      </c>
-      <c r="Q81" s="17" t="n"/>
-      <c r="R81" s="28" t="inlineStr">
-        <is>
-          <t>12 weeks</t>
-        </is>
-      </c>
-      <c r="S81" s="13" t="n"/>
-      <c r="T81" s="13" t="n">
-        <v>38</v>
-      </c>
-      <c r="U81" s="20" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="V81" s="13" t="n"/>
-      <c r="W81" s="13" t="n"/>
-      <c r="X81" s="13" t="n"/>
-      <c r="Y81" s="13" t="n"/>
-      <c r="Z81" s="13" t="n"/>
-      <c r="AA81" s="13" t="n"/>
-      <c r="AB81" s="13" t="n"/>
-      <c r="AC81" s="13" t="n"/>
-    </row>
-    <row r="82" ht="15.75" customHeight="1" s="31">
-      <c r="A82" s="13" t="inlineStr">
-        <is>
-          <t>Commonwealth Bank</t>
-        </is>
-      </c>
-      <c r="B82" s="13" t="inlineStr">
-        <is>
-          <t>Technology &amp; AI -advanced Analytics</t>
-        </is>
-      </c>
-      <c r="C82" s="13" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D82" s="13" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="E82" s="13" t="n"/>
-      <c r="F82" s="24" t="n">
-        <v>46273</v>
-      </c>
-      <c r="G82" s="29" t="n">
-        <v>46272</v>
-      </c>
-      <c r="H82" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="I82" s="13" t="n"/>
-      <c r="J82" s="13" t="n"/>
-      <c r="K82" s="13" t="n"/>
-      <c r="L82" s="13" t="n"/>
-      <c r="M82" s="13" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="N82" s="13" t="n"/>
-      <c r="O82" s="13" t="n"/>
-      <c r="P82" s="24" t="n">
-        <v>46349</v>
-      </c>
-      <c r="Q82" s="13" t="n"/>
-      <c r="R82" s="28" t="inlineStr">
-        <is>
-          <t>10 weeks</t>
-        </is>
-      </c>
-      <c r="S82" s="13" t="n"/>
-      <c r="T82" s="26" t="n">
-        <v>65000</v>
-      </c>
-      <c r="U82" s="20" t="inlineStr">
-        <is>
-          <t>1-8</t>
-        </is>
-      </c>
-      <c r="V82" s="13" t="n"/>
-      <c r="W82" s="13" t="n"/>
-      <c r="X82" s="13" t="n"/>
-      <c r="Y82" s="13" t="n"/>
-      <c r="Z82" s="13" t="n"/>
-      <c r="AA82" s="13" t="n"/>
-      <c r="AB82" s="13" t="n"/>
-      <c r="AC82" s="13" t="n"/>
-    </row>
-    <row r="83" ht="15.75" customHeight="1" s="31">
-      <c r="A83" s="32" t="inlineStr">
-        <is>
-          <t>accenture</t>
-        </is>
-      </c>
-      <c r="B83" s="32" t="inlineStr">
-        <is>
-          <t>graduate analyst technology</t>
-        </is>
-      </c>
-      <c r="C83" s="32" t="inlineStr">
-        <is>
-          <t>Graduate Program</t>
-        </is>
-      </c>
-      <c r="D83" s="32" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="F83" s="6" t="n">
-        <v>46264</v>
-      </c>
-      <c r="H83" s="32" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="M83" s="32" t="inlineStr">
-        <is>
-          <t>Withdrawn</t>
-        </is>
-      </c>
-      <c r="P83" s="6" t="inlineStr">
-        <is>
-          <t>1/19/2027 - 7/13/2027</t>
-        </is>
-      </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>70000-80000</t>
-        </is>
-      </c>
-      <c r="U83" s="7" t="inlineStr">
-        <is>
-          <t>1-45</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="15.75" customHeight="1" s="31">
-      <c r="A84" s="32" t="inlineStr">
-        <is>
-          <t>tiktok</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>business data analyst project intern (GBS)</t>
-        </is>
-      </c>
-      <c r="C84" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D84" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="n">
-        <v>46387</v>
-      </c>
-      <c r="G84" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="H84" s="13" t="inlineStr">
-        <is>
-          <t>Prosple</t>
-        </is>
-      </c>
-      <c r="M84" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="T84" t="inlineStr">
-        <is>
-          <t>2000-5000 per month</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="15.75" customHeight="1" s="31">
-      <c r="A85" s="32" t="inlineStr">
-        <is>
-          <t>Didi</t>
-        </is>
-      </c>
-      <c r="B85" s="32" t="inlineStr">
-        <is>
-          <t>operations intern</t>
-        </is>
-      </c>
-      <c r="C85" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D85" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="G85" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="M85" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="32" t="inlineStr">
-        <is>
-          <t>tencent</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Game Reaserch Development intern, engine reasearch</t>
-        </is>
-      </c>
-      <c r="C86" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D86" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="G86" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="M86" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="32" t="inlineStr">
-        <is>
-          <t>apple</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>information systems and technology</t>
-        </is>
-      </c>
-      <c r="C87" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D87" s="32" t="inlineStr">
-        <is>
-          <t>NSW</t>
-        </is>
-      </c>
-      <c r="G87" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="M87" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="32" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>student training and totation program intern</t>
-        </is>
-      </c>
-      <c r="C88" s="32" t="inlineStr">
-        <is>
-          <t>Internship</t>
-        </is>
-      </c>
-      <c r="D88" s="32" t="inlineStr">
-        <is>
-          <t>VIC</t>
-        </is>
-      </c>
-      <c r="G88" s="34" t="n">
-        <v>46277</v>
-      </c>
-      <c r="M88" s="32" t="inlineStr">
-        <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="R88" t="inlineStr">
-        <is>
-          <t>2 years</t>
-        </is>
-      </c>
-    </row>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>Attend Plan for Success workshop 29 Oct; watch for shortlist early Nov</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1" s="31"/>
+    <row r="58" ht="15.75" customHeight="1" s="31"/>
+    <row r="59" ht="15.75" customHeight="1" s="31"/>
+    <row r="60" ht="15.75" customHeight="1" s="31"/>
+    <row r="61" ht="15.75" customHeight="1" s="31"/>
+    <row r="62" ht="15.75" customHeight="1" s="31"/>
+    <row r="63" ht="15.75" customHeight="1" s="31"/>
+    <row r="64" ht="15.75" customHeight="1" s="31"/>
+    <row r="65" ht="15.75" customHeight="1" s="31"/>
+    <row r="66" ht="15.75" customHeight="1" s="31"/>
+    <row r="67" ht="15.75" customHeight="1" s="31"/>
+    <row r="68" ht="15.75" customHeight="1" s="31"/>
+    <row r="69" ht="15.75" customHeight="1" s="31"/>
+    <row r="70" ht="15.75" customHeight="1" s="31"/>
+    <row r="71" ht="15.75" customHeight="1" s="31"/>
+    <row r="72" ht="15.75" customHeight="1" s="31"/>
+    <row r="73" ht="15.75" customHeight="1" s="31"/>
+    <row r="74" ht="15.75" customHeight="1" s="31"/>
+    <row r="75" ht="15.75" customHeight="1" s="31"/>
+    <row r="76" ht="15.75" customHeight="1" s="31"/>
+    <row r="77" ht="15.75" customHeight="1" s="31"/>
+    <row r="78" ht="15.75" customHeight="1" s="31"/>
+    <row r="79" ht="15.75" customHeight="1" s="31"/>
+    <row r="80" ht="15.75" customHeight="1" s="31"/>
+    <row r="81" ht="15.75" customHeight="1" s="31"/>
+    <row r="82" ht="15.75" customHeight="1" s="31"/>
+    <row r="83" ht="15.75" customHeight="1" s="31"/>
+    <row r="84" ht="15.75" customHeight="1" s="31"/>
+    <row r="85" ht="15.75" customHeight="1" s="31"/>
   </sheetData>
-  <autoFilter ref="A1:AC94">
+  <autoFilter ref="A1:AC56">
     <sortState ref="A2:AA85">
       <sortCondition ref="M1:M85"/>
     </sortState>

</xml_diff>

<commit_message>
jobs: FDM is Project Grace Data Analyst Graduate Program, applied 27 Mar, withdrawn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6LghyMTCB4an1gFe21ULf
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -4848,15 +4848,21 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Role not recorded</t>
-        </is>
-      </c>
-      <c r="C55" s="32" t="n"/>
+          <t>Project Grace: Data Analyst Graduate Program</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t>Graduate Program</t>
+        </is>
+      </c>
       <c r="D55" s="32" t="n"/>
-      <c r="G55" s="34" t="n"/>
+      <c r="G55" s="34" t="n">
+        <v>46108</v>
+      </c>
       <c r="M55" s="32" t="inlineStr">
         <is>
-          <t>Rejected</t>
+          <t>Withdrawn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
goals: add undated plan tasks, merge vlog into brand, Mandarin and Japanese goal; AusDN withdrawn
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G6LghyMTCB4an1gFe21ULf
</commit_message>
<xml_diff>
--- a/job-applications.xlsx
+++ b/job-applications.xlsx
@@ -4888,12 +4888,7 @@
       </c>
       <c r="M56" s="32" t="inlineStr">
         <is>
-          <t>Applied</t>
-        </is>
-      </c>
-      <c r="X56" t="inlineStr">
-        <is>
-          <t>Attend Plan for Success workshop 29 Oct; watch for shortlist early Nov</t>
+          <t>Withdrawn</t>
         </is>
       </c>
     </row>

</xml_diff>